<commit_message>
Fixed image figure ratio
</commit_message>
<xml_diff>
--- a/20240519_ErCoIn_ternary_binary_combine/output/20240519_ErCoIn_ternary_binary_combine_site_pairs.xlsx
+++ b/20240519_ErCoIn_ternary_binary_combine/output/20240519_ErCoIn_ternary_binary_combine_site_pairs.xlsx
@@ -872,7 +872,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1233938.cif</t>
+          <t>1803512.cif</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -887,7 +887,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1803512.cif</t>
+          <t>1233938.cif</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1215,7 +1215,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1814810.cif</t>
+          <t>1803318.cif</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1223,14 +1223,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Deficiency without atomic mixing</t>
+          <t>Full occupancy</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1803318.cif</t>
+          <t>1814810.cif</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Full occupancy</t>
+          <t>Deficiency without atomic mixing</t>
         </is>
       </c>
     </row>

</xml_diff>